<commit_message>
added more far rules
</commit_message>
<xml_diff>
--- a/far_creation/far_CRM_uat_GBP.xlsx
+++ b/far_creation/far_CRM_uat_GBP.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Description" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LB_Details" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DNS_Entry" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FAR_Rules" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -740,7 +741,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>master0.gbpu.bank.sbi</t>
+          <t>master1.gbpu.bank.sbi</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -758,7 +759,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>master1.gbpu.bank.sbi</t>
+          <t>master2.gbpu.bank.sbi</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -963,7 +964,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>bastion1.gbpu.bank.sbi</t>
+          <t>bastion.gbpu.bank.sbi</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1111,6 +1112,453 @@
           <t>6.6.6.6</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="102" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="102" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="148" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="161" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sr.No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source IP Address</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Destination IP Address</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+1.1.1.1
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.65
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+1.1.1.1
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.65
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>TCP/1936
+TCP/9000-9999
+TCP/10249-10259
+TCP/10256
+TCP/30000-32767
+UDP/30000-32767
+UDP/30000-32767
+UDP/4789
+UDP/4500
+UDP/500
+UDP/6081
+UDP/9000-9999</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>This rule allows all traffic between the OpenShift nodes and the central bastion/mirror nodes.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+1.1.1.1
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.65
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+3.3.3.3
+4.4.4.4</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TCP/6443</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>This rule allows traffic from the OpenShift nodes to the API server on the bootstrap and master nodes.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+3.3.3.3
+4.4.4.4</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+3.3.3.3
+4.4.4.4</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TCP/2379-2380</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>This rule allows ETCD sync traffic between the bootstrap and master nodes.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+1.1.1.1
+10.177.111.65</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>10.177.111.66</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TCP/8443</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Allow all nodes to pull container images from central mirror</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1.1
+2.2.2.2
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>10.177.111.65
+1.1.1.1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>9090/TCP 
+8080/TCP</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Bastion node hosts the ignition config files and this rule is needed at the time of cluster installation to download ignition configs while creating RHCOS VMs</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+1.1.1.1
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.65
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>10.170.1.1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>6443/TCP 
+22623/TCP</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>To connect API and API-Int url from all OCP nodes</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2.2.2.2
+1.1.1.1
+3.3.3.3
+4.4.4.4
+7.7.7.7
+8.8.8.8
+9.9.9.9
+5.5.5.5
+6.6.6.6
+10.177.111.65
+10.177.111.66</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>10.170.1.2</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>443/TCP</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>To connect *.apps from all OCP nodes</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>